<commit_message>
Fill remaining 39 addresses via web research; add Address source column
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ITG_Richmond_Green_Yellow_HubSpot_Import.xlsx
+++ b/ITG_Richmond_Green_Yellow_HubSpot_Import.xlsx
@@ -380,7 +380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -394,6 +394,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,6 +453,11 @@
           <t>Phone number</t>
         </is>
       </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Address source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -504,7 +510,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -562,6 +572,11 @@
           <t>804-673-2722</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -589,6 +604,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>7130 Glen Forest Drive, Suite 101</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>23226</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>804-288-4084</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -616,6 +666,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>8700 Stony Point Parkway, Suite 120</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>23235</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>804-323-5011</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -643,6 +728,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>7202 Glen Forest Drive, Suite 200</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Henrico</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>23226</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>804-673-2024</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -670,6 +790,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>9101 Stony Point Drive</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>23235</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>804-330-9105</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -697,6 +852,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>6600 West Broad Street, Suite 300</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>804-320-4243</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -754,6 +944,11 @@
           <t>804-282-4205</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -811,6 +1006,11 @@
           <t>804-320-7139</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -868,6 +1068,11 @@
           <t>804-285-2006</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -925,6 +1130,11 @@
           <t>804-288-8204</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -982,6 +1192,11 @@
           <t>804-288-1953</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1039,6 +1254,11 @@
           <t>(804) 897-2100</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1066,6 +1286,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>400 Westhampton Station</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>23226</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>804-287-2020</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1093,6 +1348,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>7110 Forest Ave, Suite 203</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>23226</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>804-442-3558</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1145,7 +1435,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1173,6 +1467,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>12390 Three Chopt Road</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>23233</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>804-351-5432</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1225,7 +1554,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1278,7 +1611,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1306,6 +1643,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>200 North 22nd Street</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>23223</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>804-644-9590</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1333,6 +1705,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>5511 Staples Mill Road, Suite 102</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>23228</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>804-440-3700</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1360,6 +1767,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1010 N Thompson St</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>804-358-6343</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1387,6 +1829,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>517 W. Grace Street</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>23220</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>804-783-2505</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1414,6 +1891,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>4905 Dickels Road, Suite 106</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>804-712-4133</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1441,6 +1953,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1101 Hampton St</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>23220</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>804-359-4093</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1468,6 +2015,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>4825 South Laburnum Avenue</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>23231</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>804-328-1784</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1495,6 +2077,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1000 Boulders Parkway, Suite 202</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>23225</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>804-320-7881</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1552,6 +2169,11 @@
           <t>804-592-6311</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1609,6 +2231,11 @@
           <t>804-233-5481</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1636,6 +2263,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>5111 Old Midlothian Tpke</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>23224</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>804-732-9253</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1663,6 +2325,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>5004 Monument Ave</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>804-358-1150</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1690,6 +2387,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2924 Emerywood Parkway, Suite 300</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>23294</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>800-746-6768</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1717,6 +2449,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>5516 Falmouth Street, Suite 302</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>804-377-3590</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1769,7 +2536,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1822,7 +2593,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1880,6 +2655,11 @@
           <t>(804) 292-2366</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1907,6 +2687,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2369 Staples Mill Road, Suite 200</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>804-285-8206</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -1934,6 +2749,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1115 Boulders Parkway, Suite 100</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>23225</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>804-320-1339</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1991,6 +2841,11 @@
           <t>804-288-7901</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2018,6 +2873,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>6372 Mechanicsville Turnpike, Suite 103</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Mechanicsville</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>23111</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>804-379-0116</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2070,7 +2960,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2098,6 +2992,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1011 Hioaks Rd</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>23225</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>804-523-4634</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2155,6 +3084,11 @@
           <t>804-381-6252</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2182,6 +3116,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>7650 East Parham Road, MOB II Suite 210</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>23294</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>804-272-2702</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2234,7 +3203,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2287,7 +3260,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2315,6 +3292,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>204 N. Hamilton Street, Suite B</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>23221</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>877-773-3869</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2342,6 +3354,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>4900 West Marshall Street</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>804-355-5717</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2369,6 +3416,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1700 Willow Lawn Drive, Suite 210</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>804-282-9999</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2396,6 +3478,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2125 Hilliard Road</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>23228</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>804-266-9666</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -2423,6 +3540,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2125 Hilliard Road</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>23228</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>804-201-4251</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -2480,6 +3632,11 @@
           <t>804-299-3155</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2507,6 +3664,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>605 Research Rd, Suite C</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>23236</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>804-402-4420</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -2564,6 +3756,11 @@
           <t>804-622-5852</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -2621,6 +3818,11 @@
           <t>804-421-9326</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -2673,7 +3875,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -2731,6 +3937,11 @@
           <t>804-276-2800</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -2783,7 +3994,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -2836,7 +4051,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -2889,7 +4108,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -2942,7 +4165,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -2970,6 +4197,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>14653 Mountain Rd</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Glen Allen</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>23059</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>804-205-0379</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3022,7 +4284,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3080,6 +4346,11 @@
           <t>804-410-3300</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3132,7 +4403,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3160,6 +4435,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>9520 Bird Dog Dr</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Mechanicsville</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>23116</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>804-559-5417</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3217,6 +4527,11 @@
           <t>804-594-6667</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3269,7 +4584,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -3327,6 +4646,11 @@
           <t>804-798-1477</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3379,7 +4703,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3432,7 +4760,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -3490,6 +4822,11 @@
           <t>804-328-0444</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -3542,7 +4879,11 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -3600,6 +4941,11 @@
           <t>(804) 423-8372</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -3627,6 +4973,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>4915 Fitzhugh Avenue</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>804-562-5777</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -3654,6 +5035,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>7001 Forest Avenue, Suite 300</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>23230</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>804-420-1212</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -3681,6 +5097,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>7605 Forest Ave, Suite 211</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>23229</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>804-282-3114</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -3708,6 +5159,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>PO Box 13526</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>23225</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>804-276-9364</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -3735,6 +5221,41 @@
           <t>https://github.com/psdwizzard/Lists</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2810 North Parham Road, Suite 120</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>23294</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>804-288-1881</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Web research</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -3760,6 +5281,41 @@
       <c r="E81" s="7" t="inlineStr">
         <is>
           <t>https://github.com/psdwizzard/Lists</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>9221 Forest Hill Avenue</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>23235</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>804-355-0300</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Web research</t>
         </is>
       </c>
     </row>
@@ -3876,7 +5432,6 @@
           <t>23226</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4586,7 +6141,6 @@
           <t>23294</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4624,7 +6178,6 @@
           <t>23230</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4662,7 +6215,6 @@
           <t>23113</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4700,7 +6252,6 @@
           <t>23233</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4738,7 +6289,6 @@
           <t>23236</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4776,7 +6326,6 @@
           <t>23236</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4814,7 +6363,6 @@
           <t>23233</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4852,7 +6400,6 @@
           <t>23230</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4890,7 +6437,6 @@
           <t>23116</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4928,7 +6474,6 @@
           <t>23233</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4966,7 +6511,6 @@
           <t>23114</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5004,7 +6548,6 @@
           <t>23235</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5084,7 +6627,6 @@
           <t>23230</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5122,7 +6664,6 @@
           <t>23229</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5244,7 +6785,6 @@
           <t>23116</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5282,7 +6822,6 @@
           <t>23060</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5320,7 +6859,6 @@
           <t>23219</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5358,7 +6896,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5396,7 +6933,6 @@
           <t>23220</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5434,7 +6970,6 @@
           <t>23060</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5472,7 +7007,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5510,7 +7044,6 @@
           <t>23220</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5548,7 +7081,6 @@
           <t>23060</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5712,7 +7244,6 @@
           <t>23832</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5792,7 +7323,6 @@
           <t>23832</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5830,7 +7360,6 @@
           <t>23229</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5952,7 +7481,6 @@
           <t>23229</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5990,7 +7518,6 @@
           <t>23221</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6028,7 +7555,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6066,7 +7592,6 @@
           <t>22401</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6104,7 +7629,6 @@
           <t>23233</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6142,7 +7666,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6306,7 +7829,6 @@
           <t>23236</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6386,7 +7908,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6424,7 +7945,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6462,7 +7982,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6500,7 +8019,6 @@
           <t>23112</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6538,7 +8056,6 @@
           <t>23111</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6576,7 +8093,6 @@
           <t>23228</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6614,7 +8130,6 @@
           <t>23228</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6694,7 +8209,6 @@
           <t>23230</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6732,7 +8246,6 @@
           <t>23230</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6770,7 +8283,6 @@
           <t>23226</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6850,7 +8362,6 @@
           <t>23059</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6888,7 +8399,6 @@
           <t>23226</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7010,7 +8520,6 @@
           <t>23234</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7090,7 +8599,6 @@
           <t>23005</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7128,7 +8636,6 @@
           <t>23005</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7166,7 +8673,6 @@
           <t>23227</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7204,7 +8710,6 @@
           <t>23219</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7284,7 +8789,6 @@
           <t>23223</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7322,7 +8826,6 @@
           <t>23223</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7360,7 +8863,6 @@
           <t>23223</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7398,7 +8900,6 @@
           <t>23832</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7478,7 +8979,6 @@
           <t>23114</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>